<commit_message>
Greet with [name], not HubSpot's token
The emails open "Hi [name]," and the welcome email "Welcome [name]!", in
the templates, the page's own assembly, the workbook and the reference
renders, in place of the personalisation token, which is added when the
email is built in HubSpot. The page no longer needs to dress the token up.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
+++ b/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Hi {{ personalization_token('contact.firstname', 'there') }},</t>
+          <t>Hi [name],</t>
         </is>
       </c>
       <c r="C32" s="10">
@@ -2188,7 +2188,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45" ht="16" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
           <t>email · welcome · 1</t>
@@ -2196,7 +2196,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>Welcome {{ personalization_token('contact.firstname', 'to Avant Arte') }}!</t>
+          <t>Welcome [name]!</t>
         </is>
       </c>
       <c r="C45" s="10">

</xml_diff>

<commit_message>
No footer line in the emails
The templates, the page, the workbook and the docs drop the footer tagline.
The reference renders are brought up to date with the templates, tweets included.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KCpXfXvgVaMZkSdhMYLgwy
</commit_message>
<xml_diff>
--- a/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
+++ b/tool/release-copy-aiweiwei-embroidery-tl-26.xlsx
@@ -1538,7 +1538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2527,28 +2527,28 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>email · halfway · footer</t>
+          <t>email · 5 days · headline</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>There's still time to add {a_unit} to your collection.</t>
+          <t>2 days down, 5 days to go</t>
         </is>
       </c>
       <c r="C67" s="10">
-        <f>SUBSTITUTE(B67,"{a_unit}",Inputs!$B$49)</f>
+        <f>B67</f>
         <v/>
       </c>
     </row>
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>email · 5 days · headline</t>
+          <t>email · 3 days · headline</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>2 days down, 5 days to go</t>
+          <t>Three days left to collect</t>
         </is>
       </c>
       <c r="C68" s="10">
@@ -2556,221 +2556,221 @@
         <v/>
       </c>
     </row>
-    <row r="69" ht="16" customHeight="1">
+    <row r="69" ht="32" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · headline</t>
+          <t>email · 3 days · 1</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>Three days left to collect</t>
+          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C69" s="10">
-        <f>B69</f>
+        <f>SUBSTITUTE(SUBSTITUTE(B69,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$74)</f>
         <v/>
       </c>
     </row>
     <row r="70" ht="32" customHeight="1">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>email · 3 days · 1</t>
+          <t>email · 3 days · 2</t>
         </is>
       </c>
       <c r="B70" s="8" t="inlineStr">
         <is>
-          <t>There are just three days left to collect {collect_phrase} by {artist}.</t>
+          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C70" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B70,"{artist}",Inputs!$B$4),"{collect_phrase}",Inputs!$B$74)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" ht="32" customHeight="1">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>email · 3 days · 2</t>
-        </is>
-      </c>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>Click the link to collect before {close_time} on {close_weekday}, {close_date_dd}.</t>
-        </is>
-      </c>
-      <c r="C71" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B71,"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72" ht="16" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B70,"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · last chance</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="48" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>email · days to go · footer</t>
+          <t>email · last chance, timed · 1</t>
         </is>
       </c>
       <c r="B72" s="8" t="inlineStr">
         <is>
-          <t>Add {a_unit} to your collection</t>
+          <t>It's now or never for our {ordinal} collaboration with {collab_with} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C72" s="10">
-        <f>SUBSTITUTE(B72,"{a_unit}",Inputs!$B$49)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · last chance</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="48" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B72,"{collab_with}",Inputs!$B$5),"{collect_phrase}",Inputs!$B$74),"{ordinal}",Inputs!$B$10),"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="32" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>email · last chance, timed · 2</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>After this time, the edition size{each_artwork} will be confirmed, and the {work_word} will no longer be available to purchase.</t>
+        </is>
+      </c>
+      <c r="C73" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(B73,"{each_artwork}",Inputs!$B$79),"{work_word}",Inputs!$B$80)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="32" customHeight="1">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 1</t>
+          <t>email · last chance, draw · 1</t>
         </is>
       </c>
       <c r="B74" s="8" t="inlineStr">
         <is>
-          <t>It's now or never for our {ordinal} collaboration with {collab_with} – {collect_phrase} will be available to order until {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
         </is>
       </c>
       <c r="C74" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74,"{collab_with}",Inputs!$B$5),"{collect_phrase}",Inputs!$B$74),"{ordinal}",Inputs!$B$10),"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B74,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$52),"{collect_phrase}",Inputs!$B$74)</f>
         <v/>
       </c>
     </row>
     <row r="75" ht="32" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, timed · 2</t>
+          <t>email · last chance, draw · 2</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>After this time, the edition size{each_artwork} will be confirmed, and the {work_word} will no longer be available to purchase.</t>
+          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
         </is>
       </c>
       <c r="C75" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B75,"{each_artwork}",Inputs!$B$79),"{work_word}",Inputs!$B$80)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" ht="32" customHeight="1">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>email · last chance, draw · 1</t>
-        </is>
-      </c>
-      <c r="B76" s="8" t="inlineStr">
-        <is>
-          <t>This is your final opportunity to enter the draw for {work_email}, {collect_phrase} by {artist}.</t>
-        </is>
-      </c>
-      <c r="C76" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B76,"{artist}",Inputs!$B$4),"{work_email}",Inputs!$B$52),"{collect_phrase}",Inputs!$B$74)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" ht="32" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B75,"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · surveys (LE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="16" customHeight="1">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>email · last chance, draw · 2</t>
+          <t>email · first-time survey · subject</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>For a chance to collect, click the link below to enter the draw. The draw closes at {close_time} on {close_weekday}, {close_date_dd}.</t>
+          <t>Congratulations on your first Avant Arte edition</t>
         </is>
       </c>
       <c r="C77" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B77,"{close_time}",Inputs!$B$71),"{close_weekday}",Inputs!$B$72),"{close_date_dd}",Inputs!$B$73)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · surveys (LE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="16" customHeight="1">
+        <f>B77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>email · first-time survey · 1</t>
+        </is>
+      </c>
+      <c r="B78" s="8" t="inlineStr">
+        <is>
+          <t>Thank you for adding our collaboration with {collab_with} to your collection. Great choice!</t>
+        </is>
+      </c>
+      <c r="C78" s="10">
+        <f>SUBSTITUTE(B78,"{collab_with}",Inputs!$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="48" customHeight="1">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · subject</t>
+          <t>email · first-time survey · 2</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>Congratulations on your first Avant Arte edition</t>
+          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
         </is>
       </c>
       <c r="C79" s="10">
-        <f>B79</f>
+        <f>SUBSTITUTE(B79,"{advisor}",Inputs!$B$24)</f>
         <v/>
       </c>
     </row>
     <row r="80" ht="32" customHeight="1">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 1</t>
+          <t>email · first-time survey · 3</t>
         </is>
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>Thank you for adding our collaboration with {collab_with} to your collection. Great choice!</t>
+          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
         </is>
       </c>
       <c r="C80" s="10">
-        <f>SUBSTITUTE(B80,"{collab_with}",Inputs!$B$5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81" ht="48" customHeight="1">
+        <f>B80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="16" customHeight="1">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 2</t>
+          <t>email · first-time survey · 4</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>I'm {advisor}, an art advisor at Avant Arte. I'm here to connect collectors with artists by making suggestions, answering questions and offering early access to our collaborations.</t>
+          <t>Any questions? Reply to this email.</t>
         </is>
       </c>
       <c r="C81" s="10">
-        <f>SUBSTITUTE(B81,"{advisor}",Inputs!$B$24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82" ht="32" customHeight="1">
+        <f>B81</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="48" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 3</t>
+          <t>email · non-purchaser survey · 1</t>
         </is>
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>If you have two minutes to complete a short survey about your collecting journey to date, your responses will help guide my recommendations.</t>
+          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {collab_with}, we'd love your feedback.</t>
         </is>
       </c>
       <c r="C82" s="10">
-        <f>B82</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83" ht="16" customHeight="1">
+        <f>SUBSTITUTE(B82,"{collab_with}",Inputs!$B$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" ht="32" customHeight="1">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>email · first-time survey · 4</t>
+          <t>email · non-purchaser survey · 2</t>
         </is>
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>Any questions? Reply to this email.</t>
+          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
         </is>
       </c>
       <c r="C83" s="10">
@@ -2781,28 +2781,28 @@
     <row r="84" ht="48" customHeight="1">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 1</t>
+          <t>email · non-purchaser survey · 3</t>
         </is>
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>As someone who registered for updates but ultimately decided not to enter the draw for our collaboration with {collab_with}, we'd love your feedback.</t>
+          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
         </is>
       </c>
       <c r="C84" s="10">
-        <f>SUBSTITUTE(B84,"{collab_with}",Inputs!$B$5)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85" ht="32" customHeight="1">
+        <f>B84</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="16" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · 2</t>
+          <t>email · non-purchaser survey · terms</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>This two-minute survey will guide our future collaborations and help us recommend the right artists and editions for your collection.</t>
+          <t>You can read the terms here.</t>
         </is>
       </c>
       <c r="C85" s="10">
@@ -2810,106 +2810,58 @@
         <v/>
       </c>
     </row>
-    <row r="86" ht="48" customHeight="1">
-      <c r="A86" s="4" t="inlineStr">
-        <is>
-          <t>email · non-purchaser survey · 3</t>
-        </is>
-      </c>
-      <c r="B86" s="8" t="inlineStr">
-        <is>
-          <t>As a thank you for taking part in the survey and helping us improve the collector experience, you'll be entered into a draw to win a €500 Avant Arte gift card.</t>
-        </is>
-      </c>
-      <c r="C86" s="10">
-        <f>B86</f>
-        <v/>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>EMAILS · monthly preview</t>
+        </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · terms</t>
+          <t>email · monthly preview · opener</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>You can read the terms here.</t>
+          <t>From {collab_with} comes {work_intro}{support}.</t>
         </is>
       </c>
       <c r="C87" s="10">
-        <f>B87</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88" ht="16" customHeight="1">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B87,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$54),"{support}",Inputs!$B$55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" ht="32" customHeight="1">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>email · non-purchaser survey · footer</t>
+          <t>email · monthly preview · when, draw</t>
         </is>
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>What can we do better?</t>
+          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
         </is>
       </c>
       <c r="C88" s="10">
-        <f>B88</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="3" t="inlineStr">
-        <is>
-          <t>EMAILS · monthly preview</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="4" t="inlineStr">
-        <is>
-          <t>email · monthly preview · opener</t>
-        </is>
-      </c>
-      <c r="B90" s="8" t="inlineStr">
-        <is>
-          <t>From {collab_with} comes {work_intro}{support}.</t>
-        </is>
-      </c>
-      <c r="C90" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B90,"{collab_with}",Inputs!$B$5),"{work_intro}",Inputs!$B$54),"{support}",Inputs!$B$55)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="91" ht="32" customHeight="1">
-      <c r="A91" s="4" t="inlineStr">
-        <is>
-          <t>email · monthly preview · when, draw</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="inlineStr">
-        <is>
-          <t>The edition will be allocated by a randomised draw, which closes at {close_time} on {close_date}.</t>
-        </is>
-      </c>
-      <c r="C91" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(B91,"{close_date}",Inputs!$B$70),"{close_time}",Inputs!$B$71)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92" ht="32" customHeight="1">
-      <c r="A92" s="4" t="inlineStr">
+        <f>SUBSTITUTE(SUBSTITUTE(B88,"{close_date}",Inputs!$B$70),"{close_time}",Inputs!$B$71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="32" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
         <is>
           <t>email · monthly preview · when, timed</t>
         </is>
       </c>
-      <c r="B92" s="8" t="inlineStr">
+      <c r="B89" s="8" t="inlineStr">
         <is>
           <t>The edition will be available to collect for {window} only, from {launch_time} on {launch_weekday}, {launch_date_dd}.</t>
         </is>
       </c>
-      <c r="C92" s="10">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B92,"{window}",Inputs!$B$19),"{launch_time}",Inputs!$B$67),"{launch_weekday}",Inputs!$B$68),"{launch_date_dd}",Inputs!$B$69)</f>
+      <c r="C89" s="10">
+        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(B89,"{window}",Inputs!$B$19),"{launch_time}",Inputs!$B$67),"{launch_weekday}",Inputs!$B$68),"{launch_date_dd}",Inputs!$B$69)</f>
         <v/>
       </c>
     </row>
@@ -3639,7 +3591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3654,9 +3606,8 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="96" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="96" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3736,15 +3687,10 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Footer</t>
+          <t>Full email, ready to paste</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
-        <is>
-          <t>Full email, ready to paste</t>
-        </is>
-      </c>
-      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Characters</t>
         </is>
@@ -3801,15 +3747,11 @@
         <v/>
       </c>
       <c r="M4" s="11">
-        <f>IF($D4&lt;&gt;"yes","",IF(Inputs!$B$18="draw","Collect "&amp;Inputs!$B$74,"Launching "&amp;Inputs!$B$66))</f>
+        <f>IF(D4&lt;&gt;"yes",D4,IF(E4="","","Subject: "&amp;E4)&amp;IF(F4="","",CHAR(10)&amp;"Preview: "&amp;F4)&amp;IF(G4="","",CHAR(10)&amp;"Kicker: "&amp;G4)&amp;IF(H4="","",CHAR(10)&amp;"Headline: "&amp;H4)&amp;IF(I4="","",IF(E4&amp;F4&amp;G4&amp;H4="","",CHAR(10)&amp;CHAR(10))&amp;I4)&amp;IF(J4="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J4)&amp;IF(K4="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K4)&amp;IF(L4="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L4))</f>
         <v/>
       </c>
       <c r="N4" s="11">
-        <f>IF(D4&lt;&gt;"yes",D4,IF(E4="","","Subject: "&amp;E4)&amp;IF(F4="","",CHAR(10)&amp;"Preview: "&amp;F4)&amp;IF(G4="","",CHAR(10)&amp;"Kicker: "&amp;G4)&amp;IF(H4="","",CHAR(10)&amp;"Headline: "&amp;H4)&amp;IF(I4="","",IF(E4&amp;F4&amp;G4&amp;H4="","",CHAR(10)&amp;CHAR(10))&amp;I4)&amp;IF(J4="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J4)&amp;IF(K4="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K4)&amp;IF(L4="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L4)&amp;IF(M4="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M4))</f>
-        <v/>
-      </c>
-      <c r="O4" s="11">
-        <f>LEN(N4)</f>
+        <f>LEN(M4)</f>
         <v/>
       </c>
     </row>
@@ -3864,15 +3806,11 @@
         <v/>
       </c>
       <c r="M5" s="11">
-        <f>IF($D5&lt;&gt;"yes","","Where the art world is more accessible")</f>
+        <f>IF(D5&lt;&gt;"yes",D5,IF(E5="","","Subject: "&amp;E5)&amp;IF(F5="","",CHAR(10)&amp;"Preview: "&amp;F5)&amp;IF(G5="","",CHAR(10)&amp;"Kicker: "&amp;G5)&amp;IF(H5="","",CHAR(10)&amp;"Headline: "&amp;H5)&amp;IF(I5="","",IF(E5&amp;F5&amp;G5&amp;H5="","",CHAR(10)&amp;CHAR(10))&amp;I5)&amp;IF(J5="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J5)&amp;IF(K5="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K5)&amp;IF(L5="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L5))</f>
         <v/>
       </c>
       <c r="N5" s="11">
-        <f>IF(D5&lt;&gt;"yes",D5,IF(E5="","","Subject: "&amp;E5)&amp;IF(F5="","",CHAR(10)&amp;"Preview: "&amp;F5)&amp;IF(G5="","",CHAR(10)&amp;"Kicker: "&amp;G5)&amp;IF(H5="","",CHAR(10)&amp;"Headline: "&amp;H5)&amp;IF(I5="","",IF(E5&amp;F5&amp;G5&amp;H5="","",CHAR(10)&amp;CHAR(10))&amp;I5)&amp;IF(J5="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J5)&amp;IF(K5="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K5)&amp;IF(L5="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L5)&amp;IF(M5="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M5))</f>
-        <v/>
-      </c>
-      <c r="O5" s="11">
-        <f>LEN(N5)</f>
+        <f>LEN(M5)</f>
         <v/>
       </c>
     </row>
@@ -3927,15 +3865,11 @@
         <v/>
       </c>
       <c r="M6" s="11">
-        <f>IF($D6&lt;&gt;"yes","","24 hours ahead of the public launch")</f>
+        <f>IF(D6&lt;&gt;"yes",D6,IF(E6="","","Subject: "&amp;E6)&amp;IF(F6="","",CHAR(10)&amp;"Preview: "&amp;F6)&amp;IF(G6="","",CHAR(10)&amp;"Kicker: "&amp;G6)&amp;IF(H6="","",CHAR(10)&amp;"Headline: "&amp;H6)&amp;IF(I6="","",IF(E6&amp;F6&amp;G6&amp;H6="","",CHAR(10)&amp;CHAR(10))&amp;I6)&amp;IF(J6="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J6)&amp;IF(K6="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K6)&amp;IF(L6="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L6))</f>
         <v/>
       </c>
       <c r="N6" s="11">
-        <f>IF(D6&lt;&gt;"yes",D6,IF(E6="","","Subject: "&amp;E6)&amp;IF(F6="","",CHAR(10)&amp;"Preview: "&amp;F6)&amp;IF(G6="","",CHAR(10)&amp;"Kicker: "&amp;G6)&amp;IF(H6="","",CHAR(10)&amp;"Headline: "&amp;H6)&amp;IF(I6="","",IF(E6&amp;F6&amp;G6&amp;H6="","",CHAR(10)&amp;CHAR(10))&amp;I6)&amp;IF(J6="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J6)&amp;IF(K6="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K6)&amp;IF(L6="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L6)&amp;IF(M6="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M6))</f>
-        <v/>
-      </c>
-      <c r="O6" s="11">
-        <f>LEN(N6)</f>
+        <f>LEN(M6)</f>
         <v/>
       </c>
     </row>
@@ -3990,15 +3924,11 @@
         <v/>
       </c>
       <c r="M7" s="11">
-        <f>IF($D7&lt;&gt;"yes","","24 hours ahead of the public launch")</f>
+        <f>IF(D7&lt;&gt;"yes",D7,IF(E7="","","Subject: "&amp;E7)&amp;IF(F7="","",CHAR(10)&amp;"Preview: "&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;"Kicker: "&amp;G7)&amp;IF(H7="","",CHAR(10)&amp;"Headline: "&amp;H7)&amp;IF(I7="","",IF(E7&amp;F7&amp;G7&amp;H7="","",CHAR(10)&amp;CHAR(10))&amp;I7)&amp;IF(J7="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J7)&amp;IF(K7="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K7)&amp;IF(L7="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L7))</f>
         <v/>
       </c>
       <c r="N7" s="11">
-        <f>IF(D7&lt;&gt;"yes",D7,IF(E7="","","Subject: "&amp;E7)&amp;IF(F7="","",CHAR(10)&amp;"Preview: "&amp;F7)&amp;IF(G7="","",CHAR(10)&amp;"Kicker: "&amp;G7)&amp;IF(H7="","",CHAR(10)&amp;"Headline: "&amp;H7)&amp;IF(I7="","",IF(E7&amp;F7&amp;G7&amp;H7="","",CHAR(10)&amp;CHAR(10))&amp;I7)&amp;IF(J7="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J7)&amp;IF(K7="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K7)&amp;IF(L7="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L7)&amp;IF(M7="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M7))</f>
-        <v/>
-      </c>
-      <c r="O7" s="11">
-        <f>LEN(N7)</f>
+        <f>LEN(M7)</f>
         <v/>
       </c>
     </row>
@@ -4053,15 +3983,11 @@
         <v/>
       </c>
       <c r="M8" s="11">
-        <f>IF($D8&lt;&gt;"yes","",IF(Inputs!$B$18="draw","Especially for you.","24 hours ahead of the public launch"))</f>
+        <f>IF(D8&lt;&gt;"yes",D8,IF(E8="","","Subject: "&amp;E8)&amp;IF(F8="","",CHAR(10)&amp;"Preview: "&amp;F8)&amp;IF(G8="","",CHAR(10)&amp;"Kicker: "&amp;G8)&amp;IF(H8="","",CHAR(10)&amp;"Headline: "&amp;H8)&amp;IF(I8="","",IF(E8&amp;F8&amp;G8&amp;H8="","",CHAR(10)&amp;CHAR(10))&amp;I8)&amp;IF(J8="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J8)&amp;IF(K8="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K8)&amp;IF(L8="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L8))</f>
         <v/>
       </c>
       <c r="N8" s="11">
-        <f>IF(D8&lt;&gt;"yes",D8,IF(E8="","","Subject: "&amp;E8)&amp;IF(F8="","",CHAR(10)&amp;"Preview: "&amp;F8)&amp;IF(G8="","",CHAR(10)&amp;"Kicker: "&amp;G8)&amp;IF(H8="","",CHAR(10)&amp;"Headline: "&amp;H8)&amp;IF(I8="","",IF(E8&amp;F8&amp;G8&amp;H8="","",CHAR(10)&amp;CHAR(10))&amp;I8)&amp;IF(J8="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J8)&amp;IF(K8="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K8)&amp;IF(L8="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L8)&amp;IF(M8="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M8))</f>
-        <v/>
-      </c>
-      <c r="O8" s="11">
-        <f>LEN(N8)</f>
+        <f>LEN(M8)</f>
         <v/>
       </c>
     </row>
@@ -4116,15 +4042,11 @@
         <v/>
       </c>
       <c r="M9" s="11">
-        <f>IF($D9&lt;&gt;"yes","","Especially for you.")</f>
+        <f>IF(D9&lt;&gt;"yes",D9,IF(E9="","","Subject: "&amp;E9)&amp;IF(F9="","",CHAR(10)&amp;"Preview: "&amp;F9)&amp;IF(G9="","",CHAR(10)&amp;"Kicker: "&amp;G9)&amp;IF(H9="","",CHAR(10)&amp;"Headline: "&amp;H9)&amp;IF(I9="","",IF(E9&amp;F9&amp;G9&amp;H9="","",CHAR(10)&amp;CHAR(10))&amp;I9)&amp;IF(J9="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J9)&amp;IF(K9="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K9)&amp;IF(L9="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L9))</f>
         <v/>
       </c>
       <c r="N9" s="11">
-        <f>IF(D9&lt;&gt;"yes",D9,IF(E9="","","Subject: "&amp;E9)&amp;IF(F9="","",CHAR(10)&amp;"Preview: "&amp;F9)&amp;IF(G9="","",CHAR(10)&amp;"Kicker: "&amp;G9)&amp;IF(H9="","",CHAR(10)&amp;"Headline: "&amp;H9)&amp;IF(I9="","",IF(E9&amp;F9&amp;G9&amp;H9="","",CHAR(10)&amp;CHAR(10))&amp;I9)&amp;IF(J9="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J9)&amp;IF(K9="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K9)&amp;IF(L9="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L9)&amp;IF(M9="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M9))</f>
-        <v/>
-      </c>
-      <c r="O9" s="11">
-        <f>LEN(N9)</f>
+        <f>LEN(M9)</f>
         <v/>
       </c>
     </row>
@@ -4179,15 +4101,11 @@
         <v/>
       </c>
       <c r="M10" s="11">
-        <f>IF($D10&lt;&gt;"yes","","Collect "&amp;Inputs!$B$74)</f>
+        <f>IF(D10&lt;&gt;"yes",D10,IF(E10="","","Subject: "&amp;E10)&amp;IF(F10="","",CHAR(10)&amp;"Preview: "&amp;F10)&amp;IF(G10="","",CHAR(10)&amp;"Kicker: "&amp;G10)&amp;IF(H10="","",CHAR(10)&amp;"Headline: "&amp;H10)&amp;IF(I10="","",IF(E10&amp;F10&amp;G10&amp;H10="","",CHAR(10)&amp;CHAR(10))&amp;I10)&amp;IF(J10="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J10)&amp;IF(K10="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K10)&amp;IF(L10="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L10))</f>
         <v/>
       </c>
       <c r="N10" s="11">
-        <f>IF(D10&lt;&gt;"yes",D10,IF(E10="","","Subject: "&amp;E10)&amp;IF(F10="","",CHAR(10)&amp;"Preview: "&amp;F10)&amp;IF(G10="","",CHAR(10)&amp;"Kicker: "&amp;G10)&amp;IF(H10="","",CHAR(10)&amp;"Headline: "&amp;H10)&amp;IF(I10="","",IF(E10&amp;F10&amp;G10&amp;H10="","",CHAR(10)&amp;CHAR(10))&amp;I10)&amp;IF(J10="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J10)&amp;IF(K10="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K10)&amp;IF(L10="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L10)&amp;IF(M10="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M10))</f>
-        <v/>
-      </c>
-      <c r="O10" s="11">
-        <f>LEN(N10)</f>
+        <f>LEN(M10)</f>
         <v/>
       </c>
     </row>
@@ -4242,15 +4160,11 @@
         <v/>
       </c>
       <c r="M11" s="11">
-        <f>IF($D11&lt;&gt;"yes","",Lines!$C$67)</f>
+        <f>IF(D11&lt;&gt;"yes",D11,IF(E11="","","Subject: "&amp;E11)&amp;IF(F11="","",CHAR(10)&amp;"Preview: "&amp;F11)&amp;IF(G11="","",CHAR(10)&amp;"Kicker: "&amp;G11)&amp;IF(H11="","",CHAR(10)&amp;"Headline: "&amp;H11)&amp;IF(I11="","",IF(E11&amp;F11&amp;G11&amp;H11="","",CHAR(10)&amp;CHAR(10))&amp;I11)&amp;IF(J11="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J11)&amp;IF(K11="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K11)&amp;IF(L11="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L11))</f>
         <v/>
       </c>
       <c r="N11" s="11">
-        <f>IF(D11&lt;&gt;"yes",D11,IF(E11="","","Subject: "&amp;E11)&amp;IF(F11="","",CHAR(10)&amp;"Preview: "&amp;F11)&amp;IF(G11="","",CHAR(10)&amp;"Kicker: "&amp;G11)&amp;IF(H11="","",CHAR(10)&amp;"Headline: "&amp;H11)&amp;IF(I11="","",IF(E11&amp;F11&amp;G11&amp;H11="","",CHAR(10)&amp;CHAR(10))&amp;I11)&amp;IF(J11="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J11)&amp;IF(K11="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K11)&amp;IF(L11="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L11)&amp;IF(M11="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M11))</f>
-        <v/>
-      </c>
-      <c r="O11" s="11">
-        <f>LEN(N11)</f>
+        <f>LEN(M11)</f>
         <v/>
       </c>
     </row>
@@ -4285,7 +4199,7 @@
         <v/>
       </c>
       <c r="H12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$68)</f>
+        <f>IF($D12&lt;&gt;"yes","",Lines!$C$67)</f>
         <v/>
       </c>
       <c r="I12" s="11">
@@ -4305,15 +4219,11 @@
         <v/>
       </c>
       <c r="M12" s="11">
-        <f>IF($D12&lt;&gt;"yes","",Lines!$C$72)</f>
+        <f>IF(D12&lt;&gt;"yes",D12,IF(E12="","","Subject: "&amp;E12)&amp;IF(F12="","",CHAR(10)&amp;"Preview: "&amp;F12)&amp;IF(G12="","",CHAR(10)&amp;"Kicker: "&amp;G12)&amp;IF(H12="","",CHAR(10)&amp;"Headline: "&amp;H12)&amp;IF(I12="","",IF(E12&amp;F12&amp;G12&amp;H12="","",CHAR(10)&amp;CHAR(10))&amp;I12)&amp;IF(J12="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J12)&amp;IF(K12="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K12)&amp;IF(L12="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L12))</f>
         <v/>
       </c>
       <c r="N12" s="11">
-        <f>IF(D12&lt;&gt;"yes",D12,IF(E12="","","Subject: "&amp;E12)&amp;IF(F12="","",CHAR(10)&amp;"Preview: "&amp;F12)&amp;IF(G12="","",CHAR(10)&amp;"Kicker: "&amp;G12)&amp;IF(H12="","",CHAR(10)&amp;"Headline: "&amp;H12)&amp;IF(I12="","",IF(E12&amp;F12&amp;G12&amp;H12="","",CHAR(10)&amp;CHAR(10))&amp;I12)&amp;IF(J12="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J12)&amp;IF(K12="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K12)&amp;IF(L12="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L12)&amp;IF(M12="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M12))</f>
-        <v/>
-      </c>
-      <c r="O12" s="11">
-        <f>LEN(N12)</f>
+        <f>LEN(M12)</f>
         <v/>
       </c>
     </row>
@@ -4348,11 +4258,11 @@
         <v/>
       </c>
       <c r="H13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$69)</f>
+        <f>IF($D13&lt;&gt;"yes","",Lines!$C$68)</f>
         <v/>
       </c>
       <c r="I13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$70&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Lines!$C$71="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$71)&amp;IF(IF(Inputs!$B$26="","",Lines!$C$38)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$26="","",Lines!$C$38))))</f>
+        <f>IF($D13&lt;&gt;"yes","",(Lines!$C$69&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Lines!$C$70="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$70)&amp;IF(IF(Inputs!$B$26="","",Lines!$C$38)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$26="","",Lines!$C$38))))</f>
         <v/>
       </c>
       <c r="J13" s="11">
@@ -4368,15 +4278,11 @@
         <v/>
       </c>
       <c r="M13" s="11">
-        <f>IF($D13&lt;&gt;"yes","",Lines!$C$72)</f>
+        <f>IF(D13&lt;&gt;"yes",D13,IF(E13="","","Subject: "&amp;E13)&amp;IF(F13="","",CHAR(10)&amp;"Preview: "&amp;F13)&amp;IF(G13="","",CHAR(10)&amp;"Kicker: "&amp;G13)&amp;IF(H13="","",CHAR(10)&amp;"Headline: "&amp;H13)&amp;IF(I13="","",IF(E13&amp;F13&amp;G13&amp;H13="","",CHAR(10)&amp;CHAR(10))&amp;I13)&amp;IF(J13="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J13)&amp;IF(K13="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K13)&amp;IF(L13="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L13))</f>
         <v/>
       </c>
       <c r="N13" s="11">
-        <f>IF(D13&lt;&gt;"yes",D13,IF(E13="","","Subject: "&amp;E13)&amp;IF(F13="","",CHAR(10)&amp;"Preview: "&amp;F13)&amp;IF(G13="","",CHAR(10)&amp;"Kicker: "&amp;G13)&amp;IF(H13="","",CHAR(10)&amp;"Headline: "&amp;H13)&amp;IF(I13="","",IF(E13&amp;F13&amp;G13&amp;H13="","",CHAR(10)&amp;CHAR(10))&amp;I13)&amp;IF(J13="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J13)&amp;IF(K13="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K13)&amp;IF(L13="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L13)&amp;IF(M13="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M13))</f>
-        <v/>
-      </c>
-      <c r="O13" s="11">
-        <f>LEN(N13)</f>
+        <f>LEN(M13)</f>
         <v/>
       </c>
     </row>
@@ -4415,7 +4321,7 @@
         <v/>
       </c>
       <c r="I14" s="11">
-        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$18="draw",(Lines!$C$76&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Lines!$C$77="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$77)),(Lines!$C$74&amp;IF(Lines!$C$75="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$75)&amp;IF(IF(Inputs!$B$26="","",Lines!$C$38)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$26="","",Lines!$C$38)))))</f>
+        <f>IF($D14&lt;&gt;"yes","",IF(Inputs!$B$18="draw",(Lines!$C$74&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Lines!$C$75="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$75)),(Lines!$C$72&amp;IF(Lines!$C$73="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$73)&amp;IF(IF(Inputs!$B$26="","",Lines!$C$38)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$26="","",Lines!$C$38)))))</f>
         <v/>
       </c>
       <c r="J14" s="11">
@@ -4431,15 +4337,11 @@
         <v/>
       </c>
       <c r="M14" s="11">
-        <f>IF($D14&lt;&gt;"yes","","Time is almost up")</f>
+        <f>IF(D14&lt;&gt;"yes",D14,IF(E14="","","Subject: "&amp;E14)&amp;IF(F14="","",CHAR(10)&amp;"Preview: "&amp;F14)&amp;IF(G14="","",CHAR(10)&amp;"Kicker: "&amp;G14)&amp;IF(H14="","",CHAR(10)&amp;"Headline: "&amp;H14)&amp;IF(I14="","",IF(E14&amp;F14&amp;G14&amp;H14="","",CHAR(10)&amp;CHAR(10))&amp;I14)&amp;IF(J14="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J14)&amp;IF(K14="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K14)&amp;IF(L14="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L14))</f>
         <v/>
       </c>
       <c r="N14" s="11">
-        <f>IF(D14&lt;&gt;"yes",D14,IF(E14="","","Subject: "&amp;E14)&amp;IF(F14="","",CHAR(10)&amp;"Preview: "&amp;F14)&amp;IF(G14="","",CHAR(10)&amp;"Kicker: "&amp;G14)&amp;IF(H14="","",CHAR(10)&amp;"Headline: "&amp;H14)&amp;IF(I14="","",IF(E14&amp;F14&amp;G14&amp;H14="","",CHAR(10)&amp;CHAR(10))&amp;I14)&amp;IF(J14="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J14)&amp;IF(K14="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K14)&amp;IF(L14="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L14)&amp;IF(M14="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M14))</f>
-        <v/>
-      </c>
-      <c r="O14" s="11">
-        <f>LEN(N14)</f>
+        <f>LEN(M14)</f>
         <v/>
       </c>
     </row>
@@ -4462,7 +4364,7 @@
         <v/>
       </c>
       <c r="E15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",Lines!$C$79)</f>
+        <f>IF($D15&lt;&gt;"yes","",Lines!$C$77)</f>
         <v/>
       </c>
       <c r="F15" s="11">
@@ -4478,7 +4380,7 @@
         <v/>
       </c>
       <c r="I15" s="11">
-        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$32&amp;IF(Lines!$C$80="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$80)&amp;IF(Lines!$C$81="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$81)&amp;IF(Lines!$C$82="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$82)&amp;IF(Lines!$C$83="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$83)))</f>
+        <f>IF($D15&lt;&gt;"yes","",(Lines!$C$32&amp;IF(Lines!$C$78="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$78)&amp;IF(Lines!$C$79="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$79)&amp;IF(Lines!$C$80="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$80)&amp;IF(Lines!$C$81="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$81)))</f>
         <v/>
       </c>
       <c r="J15" s="11">
@@ -4494,15 +4396,11 @@
         <v/>
       </c>
       <c r="M15" s="11">
-        <f>""</f>
+        <f>IF(D15&lt;&gt;"yes",D15,IF(E15="","","Subject: "&amp;E15)&amp;IF(F15="","",CHAR(10)&amp;"Preview: "&amp;F15)&amp;IF(G15="","",CHAR(10)&amp;"Kicker: "&amp;G15)&amp;IF(H15="","",CHAR(10)&amp;"Headline: "&amp;H15)&amp;IF(I15="","",IF(E15&amp;F15&amp;G15&amp;H15="","",CHAR(10)&amp;CHAR(10))&amp;I15)&amp;IF(J15="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J15)&amp;IF(K15="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K15)&amp;IF(L15="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L15))</f>
         <v/>
       </c>
       <c r="N15" s="11">
-        <f>IF(D15&lt;&gt;"yes",D15,IF(E15="","","Subject: "&amp;E15)&amp;IF(F15="","",CHAR(10)&amp;"Preview: "&amp;F15)&amp;IF(G15="","",CHAR(10)&amp;"Kicker: "&amp;G15)&amp;IF(H15="","",CHAR(10)&amp;"Headline: "&amp;H15)&amp;IF(I15="","",IF(E15&amp;F15&amp;G15&amp;H15="","",CHAR(10)&amp;CHAR(10))&amp;I15)&amp;IF(J15="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J15)&amp;IF(K15="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K15)&amp;IF(L15="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L15)&amp;IF(M15="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M15))</f>
-        <v/>
-      </c>
-      <c r="O15" s="11">
-        <f>LEN(N15)</f>
+        <f>LEN(M15)</f>
         <v/>
       </c>
     </row>
@@ -4541,7 +4439,7 @@
         <v/>
       </c>
       <c r="I16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$84&amp;IF(Lines!$C$85="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$85)&amp;IF(Lines!$C$86="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$86)&amp;IF(Lines!$C$87="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$87)))</f>
+        <f>IF($D16&lt;&gt;"yes","",(Lines!$C$82&amp;IF(Lines!$C$83="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$83)&amp;IF(Lines!$C$84="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$84)&amp;IF(Lines!$C$85="","",CHAR(10)&amp;CHAR(10)&amp;Lines!$C$85)))</f>
         <v/>
       </c>
       <c r="J16" s="11">
@@ -4557,15 +4455,11 @@
         <v/>
       </c>
       <c r="M16" s="11">
-        <f>IF($D16&lt;&gt;"yes","",Lines!$C$88)</f>
+        <f>IF(D16&lt;&gt;"yes",D16,IF(E16="","","Subject: "&amp;E16)&amp;IF(F16="","",CHAR(10)&amp;"Preview: "&amp;F16)&amp;IF(G16="","",CHAR(10)&amp;"Kicker: "&amp;G16)&amp;IF(H16="","",CHAR(10)&amp;"Headline: "&amp;H16)&amp;IF(I16="","",IF(E16&amp;F16&amp;G16&amp;H16="","",CHAR(10)&amp;CHAR(10))&amp;I16)&amp;IF(J16="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J16)&amp;IF(K16="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K16)&amp;IF(L16="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L16))</f>
         <v/>
       </c>
       <c r="N16" s="11">
-        <f>IF(D16&lt;&gt;"yes",D16,IF(E16="","","Subject: "&amp;E16)&amp;IF(F16="","",CHAR(10)&amp;"Preview: "&amp;F16)&amp;IF(G16="","",CHAR(10)&amp;"Kicker: "&amp;G16)&amp;IF(H16="","",CHAR(10)&amp;"Headline: "&amp;H16)&amp;IF(I16="","",IF(E16&amp;F16&amp;G16&amp;H16="","",CHAR(10)&amp;CHAR(10))&amp;I16)&amp;IF(J16="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J16)&amp;IF(K16="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K16)&amp;IF(L16="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L16)&amp;IF(M16="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M16))</f>
-        <v/>
-      </c>
-      <c r="O16" s="11">
-        <f>LEN(N16)</f>
+        <f>LEN(M16)</f>
         <v/>
       </c>
     </row>
@@ -4604,7 +4498,7 @@
         <v/>
       </c>
       <c r="I17" s="11">
-        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$90&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Inputs!$B$64="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$64)&amp;IF(IF(Inputs!$B$18="draw",Lines!$C$91,Lines!$C$92)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$18="draw",Lines!$C$91,Lines!$C$92))))</f>
+        <f>IF($D17&lt;&gt;"yes","",(Lines!$C$87&amp;IF(Inputs!$B$36="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$36)&amp;IF(Inputs!$B$64="","",CHAR(10)&amp;CHAR(10)&amp;Inputs!$B$64)&amp;IF(IF(Inputs!$B$18="draw",Lines!$C$88,Lines!$C$89)="","",CHAR(10)&amp;CHAR(10)&amp;IF(Inputs!$B$18="draw",Lines!$C$88,Lines!$C$89))))</f>
         <v/>
       </c>
       <c r="J17" s="11">
@@ -4620,15 +4514,11 @@
         <v/>
       </c>
       <c r="M17" s="11">
-        <f>""</f>
+        <f>IF(D17&lt;&gt;"yes",D17,IF(E17="","","Subject: "&amp;E17)&amp;IF(F17="","",CHAR(10)&amp;"Preview: "&amp;F17)&amp;IF(G17="","",CHAR(10)&amp;"Kicker: "&amp;G17)&amp;IF(H17="","",CHAR(10)&amp;"Headline: "&amp;H17)&amp;IF(I17="","",IF(E17&amp;F17&amp;G17&amp;H17="","",CHAR(10)&amp;CHAR(10))&amp;I17)&amp;IF(J17="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J17)&amp;IF(K17="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K17)&amp;IF(L17="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L17))</f>
         <v/>
       </c>
       <c r="N17" s="11">
-        <f>IF(D17&lt;&gt;"yes",D17,IF(E17="","","Subject: "&amp;E17)&amp;IF(F17="","",CHAR(10)&amp;"Preview: "&amp;F17)&amp;IF(G17="","",CHAR(10)&amp;"Kicker: "&amp;G17)&amp;IF(H17="","",CHAR(10)&amp;"Headline: "&amp;H17)&amp;IF(I17="","",IF(E17&amp;F17&amp;G17&amp;H17="","",CHAR(10)&amp;CHAR(10))&amp;I17)&amp;IF(J17="","",CHAR(10)&amp;CHAR(10)&amp;"CTA: "&amp;J17)&amp;IF(K17="","",CHAR(10)&amp;CHAR(10)&amp;"Card: "&amp;K17)&amp;IF(L17="","",CHAR(10)&amp;CHAR(10)&amp;"Quote: "&amp;L17)&amp;IF(M17="","",CHAR(10)&amp;CHAR(10)&amp;"Footer: "&amp;M17))</f>
-        <v/>
-      </c>
-      <c r="O17" s="11">
-        <f>LEN(N17)</f>
+        <f>LEN(M17)</f>
         <v/>
       </c>
     </row>
@@ -4713,7 +4603,7 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Every email is: subject, preview, kicker, headline, body paragraphs, CTA, card, quote, footer. Bodies are fixed sentences from the Lines sheet with the same fragments dropped in. Halfway and 5 days to go have no body: they are image-led.</t>
+          <t>Every email is: subject, preview, kicker, headline, body paragraphs, CTA, card, quote. Bodies are fixed sentences from the Lines sheet with the same fragments dropped in. Halfway and 5 days to go have no body: they are image-led.</t>
         </is>
       </c>
     </row>

</xml_diff>